<commit_message>
Add sub-categoria from breadcrumb and improve terminal progress logging
Co-authored-by: Holiday090 <Holiday090@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Scraping_Action_Teste.xlsx
+++ b/Scraping_Action_Teste.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,25 +424,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Sub-categoria</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Descrição / Nome do artigo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Preço Regular</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Preço Promocional</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -454,23 +459,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Têxteis de casa de banho</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Toalha de praia sem areia | 90 x 180 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>9,98</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>6,99</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3222560/toalha-de-praia-sem-areia/</t>
         </is>
@@ -482,23 +492,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tapete | 120 x 180 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>18,95</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>14,95</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3220411/tapete/</t>
         </is>
@@ -510,23 +525,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Jarra de fruta | Ø 15,5 x 18 cm | Diversas variantes</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>5,95</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>4,99</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3213807/jarra-de-fruta/</t>
         </is>
@@ -538,23 +558,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Almofadas</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Almofada de campismo com memória de forma Froyak | 45 x 30 x 13 cm</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>7,99</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>5,95</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3204856/almofada-de-campismo-com-memoria-de-forma-froyak/</t>
         </is>
@@ -566,23 +591,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Têxteis de casa de banho</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Toalha de praia XL | 200 x 200 cm | diversas variantes</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>9,95</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>7,99</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/2581425/toalha-de-praia-xl/</t>
         </is>
@@ -594,23 +624,28 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Têxteis de casa de banho</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Toalha de praia em microfibra | 100 x 180 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>4,95</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>3,95</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/2574294/toalha-de-praia-em-microfibra/</t>
         </is>
@@ -622,19 +657,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Tapete com efeito de juta | 60 x 110 cm</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>12,95</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3221919/tapete-com-efeito-de-juta/</t>
         </is>
@@ -646,19 +686,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Almofadas</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Capa de almofada Manouk | 45 x 45 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>4,44</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3221868/capa-de-almofada-manouk/</t>
         </is>
@@ -672,21 +717,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Candeeiros</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Grundig</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Candeeiro de mesa Grundig | 400 lúmenes | Várias cores</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>13,95</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3221706/candeeiro-de-mesa-grundig/</t>
         </is>
@@ -700,21 +750,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Endless Scent</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Intensificador de fragrância Endless Scent Jasmim e Kumquat | 750 g</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>5,98</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3221547/intensificador-de-fragrancia-endless-scent-jasmim-e-kumquat/</t>
         </is>
@@ -726,19 +781,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
         <is>
           <t>Tabuleiro | Ø 30 x 2,5 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>4,99</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3220626/tabuleiro/</t>
         </is>
@@ -750,19 +810,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Armário de entrada | 90 x 38 x 42 cm</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>32,95</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3220594/armario-de-entrada/</t>
         </is>
@@ -774,19 +839,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roupa de cama</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Colcha deluxe | 220 x 240 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>19,95</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3220414/colcha-deluxe/</t>
         </is>
@@ -798,19 +868,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Cestos dobráveis | 4 peças | Várias cores</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>3,99</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3220232/cestos-dobraveis/</t>
         </is>
@@ -822,19 +897,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Lanterna Seasons &amp; Style | Ø 18 x 22 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>3,98</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3217694/lanterna-seasons-style/</t>
         </is>
@@ -846,19 +926,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Cesto arrumação em pelo sintético | 38 x 28 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>7,49</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3216174/cesto-arrumacao-em-pelo-sintetico/</t>
         </is>
@@ -870,19 +955,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Cortinado Chenille | 140 x 260 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>12,95</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3216074/cortinado-chenille/</t>
         </is>
@@ -894,19 +984,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
         <is>
           <t>Cesto | 30 x 20,5 x 12 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>2,29</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3215073/cesto/</t>
         </is>
@@ -918,19 +1013,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Cesto | 22 x 14 x 7 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>0,99</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3215070/cesto/</t>
         </is>
@@ -942,19 +1042,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Acessórios de casa de banho</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Cortina de duche de luxo | 180 x 200 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>5,95</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3215069/cortina-de-duche-de-luxo/</t>
         </is>
@@ -966,19 +1071,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Decoração</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Cestos suspensos | 31,5 x 31 x 12 cm | 2 un.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>4,95</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3212755/cestos-suspensos/</t>
         </is>
@@ -990,19 +1100,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Acessórios de viagem</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t>Sacos de vácuo com bomba elétrica | 3 peças</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>7,95</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3212383/sacos-de-vacuo-com-bomba-eletrica/</t>
         </is>
@@ -1014,19 +1129,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vasos e potes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Vaso Cadiz | Ø 30 cm | Várias cores</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>4,99</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3204441/vaso-cadiz/</t>
         </is>
@@ -1038,19 +1158,24 @@
           <t>Casa</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Candeeiros</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Candeeiro de secretária com mola | 10 watts | 300 lúmenes | 67,9 cm</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>9,95</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>https://www.action.com/pt-pt/p/3016614/candeeiro-de-secretaria-com-mola/</t>
         </is>

</xml_diff>